<commit_message>
Finalize modular structure, race history mapping, and pace standardization
</commit_message>
<xml_diff>
--- a/data/raw/possible_races.xlsx
+++ b/data/raw/possible_races.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/evancanfield/Documents/Projects/possible_races/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20509AF7-ECD6-A84A-B012-3E89A4125CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F12403C9-6136-7948-98C2-B8E22DFF4058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16620" yWindow="780" windowWidth="16620" windowHeight="21360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="900" windowWidth="33260" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="races" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">races!$A$1:$N$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">races!$A$1:$N$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="473" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="578" uniqueCount="390">
   <si>
     <t>State</t>
   </si>
@@ -716,9 +716,6 @@
     <t>https://ultrasignup.com/register.aspx?did=117259</t>
   </si>
   <si>
-    <t>https://ultrasignup.com/register.aspx?did=12+[@Lo+[@Latitude]</t>
-  </si>
-  <si>
     <t>https://www.superiorfalltrailrace.com/</t>
   </si>
   <si>
@@ -794,9 +791,6 @@
     <t>Mississippi Trail 50</t>
   </si>
   <si>
-    <t>https://www.badbeardevents.com/featured-races/stump-jump-50k-and-10-mile</t>
-  </si>
-  <si>
     <t>20 mile | 40 mile | 60 mile | 100 mile</t>
   </si>
   <si>
@@ -1026,13 +1020,199 @@
   </si>
   <si>
     <t>5K | 10K | Half Marathon | Marathon | 81 mile | 107 mile</t>
+  </si>
+  <si>
+    <t>OR</t>
+  </si>
+  <si>
+    <t>Oregon</t>
+  </si>
+  <si>
+    <t>Cascade Locks</t>
+  </si>
+  <si>
+    <t>Gorge Waterfalls</t>
+  </si>
+  <si>
+    <t>30K | 50K | 100K</t>
+  </si>
+  <si>
+    <t>https://www.daybreakracing.com/gorge-waterfalls</t>
+  </si>
+  <si>
+    <t>Prospect</t>
+  </si>
+  <si>
+    <t>Rogue Gorge</t>
+  </si>
+  <si>
+    <t>12K | Half Marathon | 50K | 50 mile</t>
+  </si>
+  <si>
+    <t>https://www.daybreakracing.com/rogue-gorge</t>
+  </si>
+  <si>
+    <t>OK</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
+  </si>
+  <si>
+    <t>Guthrie</t>
+  </si>
+  <si>
+    <t>Thunderbird Trail Run</t>
+  </si>
+  <si>
+    <t>5K | 12.5K | 25K | 50K | 100K</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=122420</t>
+  </si>
+  <si>
+    <t>Davis</t>
+  </si>
+  <si>
+    <t>Best Day Ever Ultra</t>
+  </si>
+  <si>
+    <t>10K | 20K | 50K | 100K</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=129331</t>
+  </si>
+  <si>
+    <t>Quanah</t>
+  </si>
+  <si>
+    <t>9K | 20K | 53K | 50 mile</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=127974</t>
+  </si>
+  <si>
+    <t>Poplar Bluff</t>
+  </si>
+  <si>
+    <t>Wolf Creek Trail Run</t>
+  </si>
+  <si>
+    <t>Half Marathon | 6K | 1.7 Mile</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=126662</t>
+  </si>
+  <si>
+    <t>Beaver Falls</t>
+  </si>
+  <si>
+    <t>Rabid Raccoon</t>
+  </si>
+  <si>
+    <t>Half Marathon | 100K  | 100 mile</t>
+  </si>
+  <si>
+    <t>https://runsignup.com/Race/PA/BeaverFalls/RabidRaccoon100</t>
+  </si>
+  <si>
+    <t>Frosty 15</t>
+  </si>
+  <si>
+    <t>15 mile | 15K</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=129693</t>
+  </si>
+  <si>
+    <t>Madison</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=126624</t>
+  </si>
+  <si>
+    <t>Pelham</t>
+  </si>
+  <si>
+    <t>Oak Mountain 50K</t>
+  </si>
+  <si>
+    <t>50K | 25K</t>
+  </si>
+  <si>
+    <t>Ozark Foothills Endurance Runs</t>
+  </si>
+  <si>
+    <t>25K | Marathon | 50K | 50 mile | 100K | 100 mile</t>
+  </si>
+  <si>
+    <t>https://www.terraintrailrunners.com/ozark-foothills.html</t>
+  </si>
+  <si>
+    <t>https://www.terraintrailrunners.com/babler-bongo-15k-trail-race15k-ruck.html</t>
+  </si>
+  <si>
+    <t>Babler Bongo 15K Trail Race</t>
+  </si>
+  <si>
+    <t>https://buckridgeburn.com/</t>
+  </si>
+  <si>
+    <t>5K | 10K | Half Marathon</t>
+  </si>
+  <si>
+    <t>Buck Ridge Burn</t>
+  </si>
+  <si>
+    <t>Gardners</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx?did=121875</t>
+  </si>
+  <si>
+    <t>https://www.badbeardevents.com/</t>
+  </si>
+  <si>
+    <t>Chupacabra 50</t>
+  </si>
+  <si>
+    <t>Deleware Trail Fest</t>
+  </si>
+  <si>
+    <t>12K | 24K</t>
+  </si>
+  <si>
+    <t>https://www.uberendurancesports.com/Delawaretrailfest.html</t>
+  </si>
+  <si>
+    <t>Marble Falls</t>
+  </si>
+  <si>
+    <t>Turkey Bend Bluebonnet Trail Run</t>
+  </si>
+  <si>
+    <t>https://runsignup.com/Race/TX/MarbleFalls/BluebonnetTrailRun?aflt_token=vkmwDmweQ4iCYn8otSOOnKQ3vCO8buOw</t>
+  </si>
+  <si>
+    <t>Bethel, OH</t>
+  </si>
+  <si>
+    <t>15 mile | 50K | 100K | 100 Mile</t>
+  </si>
+  <si>
+    <t>https://ultrasignup.com/register.aspx%60?did=132997</t>
+  </si>
+  <si>
+    <t>East Fork 100 mile / 100K / 50K / 15 mile</t>
+  </si>
+  <si>
+    <t>10K | Half Marathon | Marathon | 50K | 50 mile</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1082,6 +1262,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0D5ADB"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1104,7 +1297,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1115,6 +1308,7 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1152,10 +1346,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{04AB58A4-2CFD-4345-9794-A23A1DB3B6E7}" name="Table1" displayName="Table1" ref="A1:N65" totalsRowShown="0">
-  <autoFilter ref="A1:N65" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N64">
-    <sortCondition ref="A1:A64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{04AB58A4-2CFD-4345-9794-A23A1DB3B6E7}" name="Table1" displayName="Table1" ref="A1:N80" totalsRowShown="0">
+  <autoFilter ref="A1:N80" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N79">
+    <sortCondition ref="B1:B79"/>
   </sortState>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{C496E1E6-0BEB-1B44-989E-C7AA596C9564}" name="State"/>
@@ -1378,7 +1572,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N80"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
@@ -1406,7 +1600,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -1478,34 +1672,38 @@
         <v>203</v>
       </c>
       <c r="C3" t="s">
-        <v>125</v>
+        <v>101</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <f>MONTH(E3&amp;1)</f>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
       <c r="F3">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G3" t="s">
-        <v>126</v>
+        <v>103</v>
       </c>
       <c r="H3" t="s">
-        <v>127</v>
+        <v>104</v>
       </c>
       <c r="J3">
         <v>7</v>
       </c>
+      <c r="K3" t="s">
+        <v>105</v>
+      </c>
       <c r="L3">
-        <v>34.807521999999999</v>
+        <v>34.573129999999999</v>
       </c>
       <c r="M3">
-        <v>-86.589820000000003</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>128</v>
+        <v>-86.220597999999995</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1516,112 +1714,102 @@
         <v>203</v>
       </c>
       <c r="C4" t="s">
-        <v>101</v>
+        <v>125</v>
       </c>
       <c r="D4">
-        <f>MONTH(E4&amp;1)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="F4">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" t="s">
-        <v>103</v>
+        <v>126</v>
       </c>
       <c r="H4" t="s">
-        <v>104</v>
+        <v>127</v>
       </c>
       <c r="J4">
         <v>7</v>
       </c>
-      <c r="K4" t="s">
-        <v>105</v>
-      </c>
       <c r="L4">
-        <v>34.573129999999999</v>
+        <v>34.807521999999999</v>
       </c>
       <c r="M4">
-        <v>-86.220597999999995</v>
-      </c>
-      <c r="N4" s="2" t="s">
-        <v>106</v>
+        <v>-86.589820000000003</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="4" t="s">
-        <v>162</v>
+        <v>14</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>170</v>
+        <v>364</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>171</v>
+        <v>365</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I5" s="4"/>
+        <v>366</v>
+      </c>
       <c r="L5">
-        <v>35.288297</v>
+        <v>33.306065265203202</v>
       </c>
       <c r="M5">
-        <v>-92.286951000000002</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>172</v>
+        <v>-86.797008097221607</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A6" s="4" t="s">
-        <v>162</v>
+      <c r="A6" t="s">
+        <v>82</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>204</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>163</v>
+        <v>205</v>
+      </c>
+      <c r="C6" t="s">
+        <v>83</v>
       </c>
       <c r="D6">
-        <v>2</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>164</v>
-      </c>
-      <c r="H6" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>188</v>
+        <f>MONTH(E6&amp;1)</f>
+        <v>10</v>
+      </c>
+      <c r="E6" t="s">
+        <v>84</v>
+      </c>
+      <c r="G6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H6" t="s">
+        <v>86</v>
       </c>
       <c r="L6">
-        <v>34.537860999999999</v>
+        <v>35.249509000000003</v>
       </c>
       <c r="M6">
-        <v>-93.060249999999996</v>
-      </c>
-      <c r="N6" s="5" t="s">
-        <v>165</v>
+        <v>-111.686966</v>
+      </c>
+      <c r="N6" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1661,177 +1849,180 @@
       </c>
     </row>
     <row r="8" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" t="s">
-        <v>82</v>
+      <c r="A8" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>205</v>
-      </c>
-      <c r="C8" t="s">
-        <v>83</v>
+        <v>204</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>163</v>
       </c>
       <c r="D8">
-        <f>MONTH(E8&amp;1)</f>
-        <v>10</v>
-      </c>
-      <c r="E8" t="s">
-        <v>84</v>
-      </c>
-      <c r="G8" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" t="s">
-        <v>86</v>
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I8" s="4" t="s">
+        <v>188</v>
       </c>
       <c r="L8">
-        <v>35.249509000000003</v>
+        <v>34.537860999999999</v>
       </c>
       <c r="M8">
-        <v>-111.686966</v>
-      </c>
-      <c r="N8" t="s">
-        <v>224</v>
+        <v>-93.060249999999996</v>
+      </c>
+      <c r="N8" s="5" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A9" t="s">
-        <v>40</v>
+      <c r="A9" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>206</v>
-      </c>
-      <c r="C9" t="s">
-        <v>41</v>
+        <v>204</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>170</v>
       </c>
       <c r="D9">
-        <f>MONTH(E9&amp;1)</f>
-        <v>6</v>
-      </c>
-      <c r="E9" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9" s="6">
-        <v>37.906025999999997</v>
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9">
+        <v>2</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I9" s="4"/>
+      <c r="L9">
+        <v>35.288297</v>
       </c>
       <c r="M9">
-        <v>-122.54787899999999</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>45</v>
+        <v>-92.286951000000002</v>
+      </c>
+      <c r="N9" s="5" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A10" s="4" t="s">
+      <c r="A10" t="s">
         <v>40</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>206</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>196</v>
+      <c r="C10" t="s">
+        <v>41</v>
       </c>
       <c r="D10">
-        <v>9</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>199</v>
-      </c>
-      <c r="L10">
-        <v>38.984344823039898</v>
+        <f>MONTH(E10&amp;1)</f>
+        <v>6</v>
+      </c>
+      <c r="E10" t="s">
+        <v>42</v>
+      </c>
+      <c r="G10" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" t="s">
+        <v>44</v>
+      </c>
+      <c r="L10" s="6">
+        <v>37.906025999999997</v>
       </c>
       <c r="M10">
-        <v>38.984344823039898</v>
+        <v>-122.54787899999999</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>197</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="4" t="s">
-        <v>267</v>
+        <v>40</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>269</v>
+        <v>206</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>270</v>
+        <v>196</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F11">
         <v>1</v>
       </c>
       <c r="G11" s="4" t="s">
+        <v>198</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="L11">
+        <v>38.981408231814697</v>
+      </c>
+      <c r="M11">
+        <v>-120.094564336993</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A12" s="4" t="s">
+        <v>265</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>267</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>268</v>
+      </c>
+      <c r="D12">
+        <v>10</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>270</v>
+      </c>
+      <c r="L12">
+        <v>41.879522000000001</v>
+      </c>
+      <c r="M12">
+        <v>-72.195884000000007</v>
+      </c>
+      <c r="N12" s="2" t="s">
         <v>271</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>272</v>
-      </c>
-      <c r="L11">
-        <v>41.879522000000001</v>
-      </c>
-      <c r="M11">
-        <v>-72.195884000000007</v>
-      </c>
-      <c r="N11" s="2" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" t="s">
-        <v>129</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="C12" t="s">
-        <v>130</v>
-      </c>
-      <c r="D12">
-        <v>5</v>
-      </c>
-      <c r="E12" t="s">
-        <v>30</v>
-      </c>
-      <c r="F12">
-        <v>3</v>
-      </c>
-      <c r="G12" t="s">
-        <v>131</v>
-      </c>
-      <c r="H12" t="s">
-        <v>132</v>
-      </c>
-      <c r="J12">
-        <v>8</v>
-      </c>
-      <c r="L12">
-        <v>39.829008999999999</v>
-      </c>
-      <c r="M12">
-        <v>-75.571515000000005</v>
-      </c>
-      <c r="N12" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1842,34 +2033,34 @@
         <v>207</v>
       </c>
       <c r="C13" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="D13">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E13" t="s">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G13" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="H13" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="J13">
         <v>8</v>
       </c>
       <c r="L13">
-        <v>39.563349000000002</v>
+        <v>39.829008999999999</v>
       </c>
       <c r="M13">
-        <v>-75.721278999999996</v>
+        <v>-75.571515000000005</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -1880,7 +2071,7 @@
         <v>207</v>
       </c>
       <c r="C14" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D14">
         <v>10</v>
@@ -1889,246 +2080,249 @@
         <v>84</v>
       </c>
       <c r="F14">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G14" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="H14" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="J14">
         <v>8</v>
       </c>
       <c r="L14">
+        <v>39.563349000000002</v>
+      </c>
+      <c r="M14">
+        <v>-75.721278999999996</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A15" t="s">
+        <v>129</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="C15" t="s">
+        <v>138</v>
+      </c>
+      <c r="D15">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>84</v>
+      </c>
+      <c r="F15">
+        <v>3</v>
+      </c>
+      <c r="G15" t="s">
+        <v>139</v>
+      </c>
+      <c r="H15" t="s">
+        <v>140</v>
+      </c>
+      <c r="J15">
+        <v>8</v>
+      </c>
+      <c r="L15">
         <v>38.503215428965902</v>
       </c>
-      <c r="M14">
+      <c r="M15">
         <v>-75.094638952692307</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="N15" s="2" t="s">
         <v>141</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="4" t="s">
-        <v>292</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>294</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>295</v>
-      </c>
-      <c r="D15">
-        <v>12</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>296</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>297</v>
-      </c>
-      <c r="L15">
-        <v>30.122683093315899</v>
-      </c>
-      <c r="M15">
-        <v>-81.882608274474293</v>
-      </c>
-      <c r="N15" s="2" t="s">
-        <v>293</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="4" t="s">
-        <v>292</v>
+        <v>129</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>294</v>
+        <v>207</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>300</v>
+        <v>134</v>
       </c>
       <c r="D16">
+        <v>10</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16">
         <v>3</v>
       </c>
-      <c r="E16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="F16">
-        <v>2</v>
-      </c>
       <c r="G16" s="4" t="s">
-        <v>299</v>
+        <v>379</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>301</v>
+        <v>380</v>
       </c>
       <c r="L16">
-        <v>29.258558821513802</v>
+        <v>39.618131235885102</v>
       </c>
       <c r="M16">
-        <v>-81.681933881918994</v>
+        <v>-75.672643463456794</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>298</v>
+        <v>381</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B17" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="B17" s="4" t="s">
+      <c r="C17" s="4" t="s">
+        <v>293</v>
+      </c>
+      <c r="D17">
+        <v>12</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4" t="s">
         <v>294</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="H17" s="4" t="s">
         <v>295</v>
       </c>
-      <c r="D17">
-        <v>5</v>
-      </c>
-      <c r="E17" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17">
-        <v>2</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>302</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>303</v>
-      </c>
       <c r="L17">
-        <v>30.1224312540493</v>
+        <v>30.122683093315899</v>
       </c>
       <c r="M17">
-        <v>-81.882363825334707</v>
+        <v>-81.882608274474293</v>
       </c>
       <c r="N17" s="2" t="s">
-        <v>304</v>
+        <v>291</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B18" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>294</v>
-      </c>
       <c r="C18" s="4" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>84</v>
+        <v>11</v>
       </c>
       <c r="F18">
         <v>4</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>54</v>
+        <v>312</v>
       </c>
       <c r="L18">
-        <v>29.775124598000801</v>
+        <v>30.720986421985099</v>
       </c>
       <c r="M18">
-        <v>-82.473914728266195</v>
-      </c>
-      <c r="N18" s="2" t="s">
-        <v>306</v>
+        <v>-81.450561534488003</v>
+      </c>
+      <c r="N18" s="5" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B19" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="B19" s="4" t="s">
-        <v>294</v>
-      </c>
       <c r="C19" s="4" t="s">
-        <v>311</v>
+        <v>298</v>
+      </c>
+      <c r="D19">
+        <v>3</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>102</v>
+        <v>21</v>
       </c>
       <c r="F19">
         <v>2</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="K19" s="4" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="L19">
-        <v>30.501792962740399</v>
+        <v>29.258558821513802</v>
       </c>
       <c r="M19">
-        <v>-82.673175708148193</v>
+        <v>-81.681933881918994</v>
       </c>
       <c r="N19" s="2" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B20" s="4" t="s">
         <v>292</v>
       </c>
-      <c r="B20" s="4" t="s">
-        <v>294</v>
-      </c>
       <c r="C20" s="4" t="s">
-        <v>312</v>
+        <v>293</v>
       </c>
       <c r="D20">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="H20" s="4" t="s">
-        <v>314</v>
+        <v>301</v>
       </c>
       <c r="L20">
-        <v>30.720986421985099</v>
+        <v>30.1224312540493</v>
       </c>
       <c r="M20">
-        <v>-81.450561534488003</v>
+        <v>-81.882363825334707</v>
       </c>
       <c r="N20" s="2" t="s">
-        <v>315</v>
+        <v>302</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="4" t="s">
-        <v>184</v>
+        <v>290</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>208</v>
+        <v>292</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>186</v>
+        <v>309</v>
       </c>
       <c r="D21">
         <v>11</v>
@@ -2137,61 +2331,60 @@
         <v>102</v>
       </c>
       <c r="F21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>187</v>
+        <v>307</v>
       </c>
       <c r="H21" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="K21" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="L21">
+        <v>30.501792962740399</v>
+      </c>
+      <c r="M21">
+        <v>-82.673175708148193</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A22" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>305</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="H22" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="I21" s="4"/>
-      <c r="L21" s="4">
-        <v>42.459299092168102</v>
-      </c>
-      <c r="M21">
-        <v>-90.6640480371547</v>
-      </c>
-      <c r="N21" s="5" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" t="s">
-        <v>142</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C22" t="s">
-        <v>147</v>
-      </c>
-      <c r="D22">
-        <v>3</v>
-      </c>
-      <c r="E22" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22">
-        <v>3</v>
-      </c>
-      <c r="G22" t="s">
-        <v>148</v>
-      </c>
-      <c r="H22" t="s">
-        <v>149</v>
-      </c>
-      <c r="J22">
-        <v>10</v>
-      </c>
       <c r="L22">
-        <v>39.344932</v>
+        <v>29.775124598000801</v>
       </c>
       <c r="M22">
-        <v>-86.852144999999993</v>
+        <v>-82.473914728266195</v>
       </c>
       <c r="N22" s="2" t="s">
-        <v>150</v>
+        <v>304</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2202,31 +2395,34 @@
         <v>209</v>
       </c>
       <c r="C23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D23">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>76</v>
+        <v>21</v>
+      </c>
+      <c r="F23">
+        <v>3</v>
       </c>
       <c r="G23" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="H23" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="J23">
-        <v>8</v>
-      </c>
-      <c r="L23" s="4">
-        <v>38.4623343165783</v>
+        <v>10</v>
+      </c>
+      <c r="L23">
+        <v>39.344932</v>
       </c>
       <c r="M23">
-        <v>-85.862459795099795</v>
+        <v>-86.852144999999993</v>
       </c>
       <c r="N23" s="2" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2269,120 +2465,112 @@
     </row>
     <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>20</v>
+        <v>142</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>151</v>
       </c>
       <c r="D25">
-        <f>MONTH(E25&amp;1)</f>
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E25" t="s">
-        <v>25</v>
-      </c>
-      <c r="F25">
-        <v>1</v>
+        <v>76</v>
       </c>
       <c r="G25" t="s">
-        <v>26</v>
+        <v>152</v>
       </c>
       <c r="H25" t="s">
-        <v>27</v>
-      </c>
-      <c r="K25" t="s">
-        <v>120</v>
-      </c>
-      <c r="L25">
-        <v>37.784264999999998</v>
+        <v>153</v>
+      </c>
+      <c r="J25">
+        <v>8</v>
+      </c>
+      <c r="L25" s="4">
+        <v>38.4623343165783</v>
       </c>
       <c r="M25">
-        <v>-83.632585000000006</v>
-      </c>
-      <c r="N25" s="5" t="s">
-        <v>225</v>
+        <v>-85.862459795099795</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" t="s">
-        <v>20</v>
+      <c r="A26" s="4" t="s">
+        <v>184</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>210</v>
-      </c>
-      <c r="C26" t="s">
-        <v>117</v>
+        <v>208</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>186</v>
       </c>
       <c r="D26">
         <v>11</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="4" t="s">
         <v>102</v>
       </c>
       <c r="F26">
-        <v>2</v>
-      </c>
-      <c r="G26" t="s">
-        <v>118</v>
-      </c>
-      <c r="H26" t="s">
-        <v>119</v>
-      </c>
-      <c r="J26">
-        <v>6</v>
-      </c>
-      <c r="K26" t="s">
-        <v>120</v>
-      </c>
-      <c r="L26">
-        <v>37.781091000000004</v>
+        <v>1</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="I26" s="4"/>
+      <c r="L26" s="4">
+        <v>42.459299092168102</v>
       </c>
       <c r="M26">
-        <v>-83.689959000000002</v>
-      </c>
-      <c r="N26" s="2" t="s">
-        <v>121</v>
+        <v>-90.6640480371547</v>
+      </c>
+      <c r="N26" s="5" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A27" s="4" t="s">
+      <c r="A27" t="s">
         <v>20</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="C27" s="4" t="s">
-        <v>316</v>
+      <c r="C27" t="s">
+        <v>24</v>
       </c>
       <c r="D27">
+        <f>MONTH(E27&amp;1)</f>
         <v>4</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" t="s">
         <v>25</v>
       </c>
       <c r="F27">
-        <v>4</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>317</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>318</v>
-      </c>
-      <c r="J27">
-        <v>6</v>
-      </c>
-      <c r="L27" s="5">
-        <v>38.191333504485499</v>
-      </c>
-      <c r="M27" s="7">
-        <v>-83.431420053320096</v>
-      </c>
-      <c r="N27" s="2" t="s">
-        <v>319</v>
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
+        <v>26</v>
+      </c>
+      <c r="H27" t="s">
+        <v>27</v>
+      </c>
+      <c r="K27" t="s">
+        <v>120</v>
+      </c>
+      <c r="L27">
+        <v>37.784264999999998</v>
+      </c>
+      <c r="M27">
+        <v>-83.632585000000006</v>
+      </c>
+      <c r="N27" s="5" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2393,175 +2581,183 @@
         <v>210</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="D28">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="F28">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="J28">
-        <v>5.5</v>
-      </c>
-      <c r="L28">
-        <v>37.141310259329998</v>
-      </c>
-      <c r="M28">
-        <v>83.430232358848002</v>
+        <v>6</v>
+      </c>
+      <c r="L28" s="5">
+        <v>38.191333504485499</v>
+      </c>
+      <c r="M28" s="7">
+        <v>-83.431420053320096</v>
       </c>
       <c r="N28" s="2" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="D29">
+        <v>3</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="J29">
+        <v>5.5</v>
+      </c>
+      <c r="L29">
+        <v>37.141310259329998</v>
+      </c>
+      <c r="M29">
+        <v>83.430232358848002</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A30" t="s">
+        <v>20</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="C30" t="s">
+        <v>117</v>
+      </c>
+      <c r="D30">
+        <v>11</v>
+      </c>
+      <c r="E30" t="s">
+        <v>102</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30" t="s">
+        <v>118</v>
+      </c>
+      <c r="H30" t="s">
+        <v>119</v>
+      </c>
+      <c r="J30">
+        <v>6</v>
+      </c>
+      <c r="K30" t="s">
+        <v>120</v>
+      </c>
+      <c r="L30">
+        <v>37.781091000000004</v>
+      </c>
+      <c r="M30">
+        <v>-83.689959000000002</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A31" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B31" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="B29" s="4" t="s">
+      <c r="C31" s="4" t="s">
         <v>236</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="D31">
+        <v>12</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31" s="4" t="s">
         <v>237</v>
       </c>
-      <c r="D29">
-        <v>12</v>
-      </c>
-      <c r="E29" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29" s="4" t="s">
+      <c r="H31" s="4" t="s">
+        <v>251</v>
+      </c>
+      <c r="L31">
+        <v>30.788984200292902</v>
+      </c>
+      <c r="M31">
+        <v>-92.282911832662407</v>
+      </c>
+      <c r="N31" s="2" t="s">
         <v>238</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>253</v>
-      </c>
-      <c r="L29">
-        <v>30.788984200292902</v>
-      </c>
-      <c r="M29">
-        <v>-92.282911832662407</v>
-      </c>
-      <c r="N29" s="2" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>240</v>
-      </c>
-      <c r="D30">
-        <v>10</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F30">
-        <v>1</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="L30" s="4">
-        <v>32.535883651366603</v>
-      </c>
-      <c r="M30">
-        <v>-93.410972717249095</v>
-      </c>
-      <c r="N30" s="2" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="C31" t="s">
-        <v>29</v>
-      </c>
-      <c r="D31">
-        <f>MONTH(E31&amp;1)</f>
-        <v>5</v>
-      </c>
-      <c r="E31" t="s">
-        <v>30</v>
-      </c>
-      <c r="G31" t="s">
-        <v>31</v>
-      </c>
-      <c r="H31" t="s">
-        <v>32</v>
-      </c>
-      <c r="K31" t="s">
-        <v>33</v>
-      </c>
-      <c r="L31">
-        <v>42.305984000000002</v>
-      </c>
-      <c r="M31">
-        <v>-72.532236999999995</v>
-      </c>
-      <c r="N31" s="2" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="4" t="s">
-        <v>28</v>
+        <v>234</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>193</v>
+        <v>239</v>
       </c>
       <c r="D32">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>42</v>
+        <v>84</v>
       </c>
       <c r="F32">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>194</v>
+        <v>240</v>
       </c>
       <c r="H32" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="L32">
-        <v>42.481794999999998</v>
+        <v>252</v>
+      </c>
+      <c r="L32" s="4">
+        <v>32.535883651366603</v>
       </c>
       <c r="M32">
-        <v>-73.301186999999999</v>
-      </c>
-      <c r="N32" s="5" t="s">
-        <v>226</v>
+        <v>-93.410972717249095</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -2638,240 +2834,237 @@
     </row>
     <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="D35">
+        <v>6</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F35">
+        <v>3</v>
+      </c>
+      <c r="G35" s="4" t="s">
+        <v>194</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="L35">
+        <v>42.481794999999998</v>
+      </c>
+      <c r="M35">
+        <v>-73.301186999999999</v>
+      </c>
+      <c r="N35" s="5" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A36" t="s">
+        <v>28</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="C36" t="s">
+        <v>29</v>
+      </c>
+      <c r="D36">
+        <f>MONTH(E36&amp;1)</f>
+        <v>5</v>
+      </c>
+      <c r="E36" t="s">
+        <v>30</v>
+      </c>
+      <c r="G36" t="s">
+        <v>31</v>
+      </c>
+      <c r="H36" t="s">
+        <v>32</v>
+      </c>
+      <c r="K36" t="s">
+        <v>33</v>
+      </c>
+      <c r="L36">
+        <v>42.305984000000002</v>
+      </c>
+      <c r="M36">
+        <v>-72.532236999999995</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A37" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B35" s="4" t="s">
+      <c r="B37" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C37" t="s">
         <v>56</v>
-      </c>
-      <c r="D35">
-        <f>MONTH(E35&amp;1)</f>
-        <v>7</v>
-      </c>
-      <c r="E35" t="s">
-        <v>52</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="H35" t="s">
-        <v>57</v>
-      </c>
-      <c r="L35" s="4">
-        <v>46.453039091063701</v>
-      </c>
-      <c r="M35" s="4">
-        <v>-86.665557210347103</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A36" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>283</v>
-      </c>
-      <c r="D36">
-        <v>7</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F36">
-        <v>3</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>285</v>
-      </c>
-      <c r="H36" s="4" t="s">
-        <v>286</v>
-      </c>
-      <c r="L36">
-        <v>43.054254833541002</v>
-      </c>
-      <c r="M36">
-        <v>-85.501292315380496</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A37" t="s">
-        <v>74</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C37" t="s">
-        <v>75</v>
       </c>
       <c r="D37">
         <f>MONTH(E37&amp;1)</f>
+        <v>7</v>
+      </c>
+      <c r="E37" t="s">
+        <v>52</v>
+      </c>
+      <c r="G37" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H37" t="s">
+        <v>57</v>
+      </c>
+      <c r="L37" s="4">
+        <v>46.453039091063701</v>
+      </c>
+      <c r="M37" s="4">
+        <v>-86.665557210347103</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A38" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C38" s="4" t="s">
+        <v>281</v>
+      </c>
+      <c r="D38">
+        <v>7</v>
+      </c>
+      <c r="E38" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F38">
+        <v>3</v>
+      </c>
+      <c r="G38" s="4" t="s">
+        <v>283</v>
+      </c>
+      <c r="H38" s="4" t="s">
+        <v>284</v>
+      </c>
+      <c r="L38">
+        <v>43.054254833541002</v>
+      </c>
+      <c r="M38">
+        <v>-85.501292315380496</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A39" t="s">
+        <v>74</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C39" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39">
+        <f>MONTH(E39&amp;1)</f>
+        <v>10</v>
+      </c>
+      <c r="E39" t="s">
+        <v>84</v>
+      </c>
+      <c r="G39" t="s">
+        <v>88</v>
+      </c>
+      <c r="H39" t="s">
+        <v>89</v>
+      </c>
+      <c r="L39" s="4">
+        <v>46.661502722688297</v>
+      </c>
+      <c r="M39" s="4">
+        <v>-92.282658270523996</v>
+      </c>
+      <c r="N39" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A40" t="s">
+        <v>74</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="C40" t="s">
+        <v>75</v>
+      </c>
+      <c r="D40">
+        <f>MONTH(E40&amp;1)</f>
         <v>9</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E40" t="s">
         <v>76</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G40" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="H37" s="4" t="s">
-        <v>256</v>
-      </c>
-      <c r="I37" s="4"/>
-      <c r="K37" t="s">
+      <c r="H40" s="4" t="s">
+        <v>254</v>
+      </c>
+      <c r="I40" s="4"/>
+      <c r="K40" t="s">
         <v>78</v>
       </c>
-      <c r="L37">
+      <c r="L40">
         <v>47.540463000000003</v>
       </c>
-      <c r="M37">
+      <c r="M40">
         <v>-90.978267000000002</v>
       </c>
-      <c r="N37" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="38" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A38" t="s">
-        <v>74</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="C38" t="s">
-        <v>87</v>
-      </c>
-      <c r="D38">
-        <f>MONTH(E38&amp;1)</f>
-        <v>10</v>
-      </c>
-      <c r="E38" t="s">
-        <v>84</v>
-      </c>
-      <c r="G38" t="s">
-        <v>88</v>
-      </c>
-      <c r="H38" t="s">
-        <v>89</v>
-      </c>
-      <c r="L38" s="4">
-        <v>46.661502722688297</v>
-      </c>
-      <c r="M38" s="4">
-        <v>-92.282658270523996</v>
-      </c>
-      <c r="N38" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="39" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A39" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="D39">
-        <v>12</v>
-      </c>
-      <c r="E39" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="F39">
-        <v>2</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H39" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="I39" s="4"/>
-      <c r="K39" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="L39" s="4">
-        <v>38.551906000000002</v>
-      </c>
-      <c r="M39" s="4">
-        <v>-90.638622999999995</v>
-      </c>
-      <c r="N39" s="5" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="40" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A40" s="4" t="s">
-        <v>243</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="D40">
-        <v>9</v>
-      </c>
-      <c r="E40" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="F40">
-        <v>4</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="H40" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="L40">
-        <v>32.107823000000003</v>
-      </c>
-      <c r="M40">
-        <v>-88.697120999999996</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>248</v>
+      <c r="N40" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B41" s="4" t="s">
         <v>243</v>
       </c>
-      <c r="B41" s="4" t="s">
-        <v>244</v>
-      </c>
       <c r="C41" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="D41">
+        <v>3</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41" s="4" t="s">
         <v>250</v>
       </c>
-      <c r="D41">
-        <v>2</v>
-      </c>
-      <c r="E41" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F41">
-        <v>4</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>251</v>
-      </c>
       <c r="H41" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="L41">
         <v>31.568680000000001</v>
@@ -2880,903 +3073,1431 @@
         <v>-88.987307000000001</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="42" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A42" s="4" t="s">
-        <v>262</v>
+        <v>242</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>263</v>
+        <v>243</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>264</v>
+        <v>244</v>
       </c>
       <c r="D42">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E42" s="4" t="s">
-        <v>30</v>
+        <v>76</v>
       </c>
       <c r="F42">
         <v>4</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>265</v>
+        <v>245</v>
       </c>
       <c r="H42" s="4" t="s">
-        <v>266</v>
+        <v>246</v>
       </c>
       <c r="L42">
-        <v>41.423577761322598</v>
+        <v>32.107823000000003</v>
       </c>
       <c r="M42">
-        <v>-96.543395340635797</v>
+        <v>-88.697120999999996</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>261</v>
+        <v>247</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A43" t="s">
-        <v>59</v>
+      <c r="A43" s="4" t="s">
+        <v>242</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>217</v>
-      </c>
-      <c r="C43" t="s">
-        <v>60</v>
+        <v>243</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>362</v>
       </c>
       <c r="D43">
-        <f>MONTH(E43&amp;1)</f>
-        <v>7</v>
-      </c>
-      <c r="E43" t="s">
-        <v>52</v>
-      </c>
-      <c r="G43" t="s">
-        <v>61</v>
-      </c>
-      <c r="H43" t="s">
-        <v>62</v>
-      </c>
-      <c r="L43" s="4">
-        <v>36.708372823836598</v>
-      </c>
-      <c r="M43" s="4">
-        <v>-105.405565676064</v>
+        <v>2</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43">
+        <v>2</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="L43">
+        <v>32.465625290305503</v>
+      </c>
+      <c r="M43">
+        <v>-90.057065187102793</v>
       </c>
       <c r="N43" s="2" t="s">
-        <v>63</v>
+        <v>361</v>
       </c>
     </row>
     <row r="44" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A44" s="4" t="s">
-        <v>59</v>
+        <v>173</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="D44">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>76</v>
+        <v>174</v>
       </c>
       <c r="F44">
         <v>2</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>157</v>
+        <v>176</v>
       </c>
       <c r="H44" s="4" t="s">
-        <v>260</v>
+        <v>62</v>
       </c>
       <c r="I44" s="4"/>
-      <c r="L44">
-        <v>36.595438000000001</v>
-      </c>
-      <c r="M44">
-        <v>-105.447819</v>
+      <c r="K44" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="L44" s="4">
+        <v>38.551906000000002</v>
+      </c>
+      <c r="M44" s="4">
+        <v>-90.638622999999995</v>
       </c>
       <c r="N44" s="5" t="s">
-        <v>158</v>
+        <v>178</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A45" s="4" t="s">
-        <v>59</v>
+        <v>173</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>159</v>
+        <v>351</v>
       </c>
       <c r="D45">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="F45">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>160</v>
+        <v>352</v>
       </c>
       <c r="H45" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I45" s="4"/>
-      <c r="L45" s="4">
-        <v>35.777392185115701</v>
+        <v>353</v>
+      </c>
+      <c r="L45">
+        <v>36.750821139959797</v>
       </c>
       <c r="M45">
-        <v>-105.81082548955899</v>
+        <v>-90.4059322406832</v>
       </c>
       <c r="N45" s="2" t="s">
-        <v>161</v>
+        <v>354</v>
       </c>
     </row>
     <row r="46" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A46" s="4" t="s">
-        <v>59</v>
+        <v>173</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="D46">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>68</v>
+        <v>25</v>
       </c>
       <c r="F46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>275</v>
+        <v>367</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>276</v>
-      </c>
-      <c r="L46">
-        <v>36.406430042726697</v>
+        <v>368</v>
+      </c>
+      <c r="L46" s="4">
+        <v>38.5276605403497</v>
       </c>
       <c r="M46">
-        <v>-105.572292389526</v>
+        <v>-90.686490436578097</v>
       </c>
       <c r="N46" s="2" t="s">
-        <v>274</v>
+        <v>369</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A47" t="s">
-        <v>96</v>
+      <c r="A47" s="4" t="s">
+        <v>173</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="C47" t="s">
-        <v>97</v>
+        <v>216</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>175</v>
       </c>
       <c r="D47">
         <v>10</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E47" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="G47" t="s">
-        <v>98</v>
-      </c>
-      <c r="H47" t="s">
-        <v>257</v>
-      </c>
-      <c r="J47">
-        <v>7</v>
-      </c>
-      <c r="K47" t="s">
-        <v>99</v>
+      <c r="F47">
+        <v>4</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>371</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>104</v>
       </c>
       <c r="L47">
-        <v>38.739795000000001</v>
+        <v>38.617799328111097</v>
       </c>
       <c r="M47">
-        <v>-83.203586999999999</v>
+        <v>-90.689514775249194</v>
       </c>
       <c r="N47" s="2" t="s">
-        <v>100</v>
+        <v>370</v>
       </c>
     </row>
     <row r="48" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A48" s="4" t="s">
-        <v>96</v>
+        <v>260</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>218</v>
+        <v>261</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>179</v>
+        <v>262</v>
       </c>
       <c r="D48">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>84</v>
+        <v>30</v>
       </c>
       <c r="F48">
         <v>4</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>180</v>
+        <v>263</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="I48" s="4"/>
-      <c r="J48" s="4"/>
-      <c r="K48" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="L48" s="4">
-        <v>41.224018000000001</v>
-      </c>
-      <c r="M48" s="4">
-        <v>-81.510507000000004</v>
-      </c>
-      <c r="N48" s="5" t="s">
-        <v>183</v>
+        <v>264</v>
+      </c>
+      <c r="L48">
+        <v>41.423577761322598</v>
+      </c>
+      <c r="M48">
+        <v>-96.543395340635797</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="49" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A49" s="4" t="s">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>191</v>
+        <v>156</v>
       </c>
       <c r="D49">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="F49">
         <v>1</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>189</v>
+        <v>273</v>
       </c>
       <c r="H49" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="J49">
-        <v>6</v>
+        <v>274</v>
       </c>
       <c r="L49">
-        <v>39.320948000000001</v>
+        <v>36.406430042726697</v>
       </c>
       <c r="M49">
-        <v>-82.356718999999998</v>
-      </c>
-      <c r="N49" s="5" t="s">
-        <v>190</v>
+        <v>-105.572292389526</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>272</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A50" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C50" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="D50">
         <f>MONTH(E50&amp;1)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E50" t="s">
-        <v>68</v>
+        <v>52</v>
       </c>
       <c r="G50" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H50" t="s">
-        <v>27</v>
-      </c>
-      <c r="J50">
+        <v>62</v>
+      </c>
+      <c r="L50" s="4">
+        <v>36.708372823836598</v>
+      </c>
+      <c r="M50" s="4">
+        <v>-105.405565676064</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A51" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C51" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="D51">
+        <v>10</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="F51">
+        <v>2</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="H51" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="I51" s="4"/>
+      <c r="L51" s="4">
+        <v>35.777392185115701</v>
+      </c>
+      <c r="M51">
+        <v>-105.81082548955899</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A52" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="C52" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="D52">
         <v>9</v>
       </c>
-      <c r="L50">
-        <v>41.345925000000001</v>
-      </c>
-      <c r="M50">
-        <v>-79.218463</v>
-      </c>
-      <c r="N50" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="51" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A51" t="s">
-        <v>66</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="C51" t="s">
-        <v>79</v>
-      </c>
-      <c r="D51">
-        <f>MONTH(E51&amp;1)</f>
-        <v>9</v>
-      </c>
-      <c r="E51" t="s">
+      <c r="E52" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="G51" t="s">
-        <v>80</v>
-      </c>
-      <c r="H51" t="s">
+      <c r="F52">
+        <v>2</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="H52" s="4" t="s">
         <v>258</v>
       </c>
-      <c r="J51">
-        <v>9</v>
-      </c>
-      <c r="L51">
-        <v>41.134135000000001</v>
-      </c>
-      <c r="M51">
-        <v>-77.420109999999994</v>
-      </c>
-      <c r="N51" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="52" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A52" t="s">
-        <v>66</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>219</v>
-      </c>
-      <c r="C52" t="s">
-        <v>90</v>
-      </c>
-      <c r="D52">
-        <f>MONTH(E52&amp;1)</f>
-        <v>10</v>
-      </c>
-      <c r="E52" t="s">
-        <v>84</v>
-      </c>
-      <c r="G52" t="s">
-        <v>91</v>
-      </c>
-      <c r="H52" t="s">
-        <v>54</v>
-      </c>
-      <c r="J52">
-        <v>9</v>
-      </c>
+      <c r="I52" s="4"/>
       <c r="L52">
-        <v>41.363957999999997</v>
+        <v>36.595438000000001</v>
       </c>
       <c r="M52">
-        <v>-77.356221000000005</v>
-      </c>
-      <c r="N52" s="2" t="s">
-        <v>92</v>
+        <v>-105.447819</v>
+      </c>
+      <c r="N52" s="5" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="53" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A53" t="s">
-        <v>46</v>
+      <c r="A53" s="4" t="s">
+        <v>322</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="C53" t="s">
-        <v>47</v>
+        <v>323</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>326</v>
       </c>
       <c r="D53">
-        <f>MONTH(E53&amp;1)</f>
         <v>6</v>
       </c>
-      <c r="E53" t="s">
+      <c r="E53" s="4" t="s">
         <v>42</v>
       </c>
+      <c r="F53">
+        <v>4</v>
+      </c>
       <c r="G53" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="H53" t="s">
-        <v>49</v>
-      </c>
-      <c r="L53" s="4">
-        <v>41.441013820781301</v>
+        <v>325</v>
+      </c>
+      <c r="H53" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="L53">
+        <v>46.913974694365898</v>
       </c>
       <c r="M53">
-        <v>-71.463694190880901</v>
-      </c>
-      <c r="N53" t="s">
-        <v>229</v>
+        <v>-103.52377003853699</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>324</v>
       </c>
     </row>
     <row r="54" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A54" t="s">
-        <v>46</v>
+      <c r="A54" s="4" t="s">
+        <v>96</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>220</v>
-      </c>
-      <c r="C54" t="s">
-        <v>93</v>
+        <v>218</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>191</v>
       </c>
       <c r="D54">
-        <f>MONTH(E54&amp;1)</f>
-        <v>10</v>
-      </c>
-      <c r="E54" t="s">
-        <v>84</v>
-      </c>
-      <c r="G54" t="s">
-        <v>94</v>
-      </c>
-      <c r="H54" t="s">
-        <v>95</v>
+        <v>4</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F54">
+        <v>1</v>
+      </c>
+      <c r="G54" s="4" t="s">
+        <v>189</v>
+      </c>
+      <c r="H54" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="J54">
+        <v>6</v>
       </c>
       <c r="L54">
-        <v>41.361185752662699</v>
+        <v>39.320948000000001</v>
       </c>
       <c r="M54">
-        <v>-71.4813502625707</v>
-      </c>
-      <c r="N54" t="s">
-        <v>230</v>
+        <v>-82.356718999999998</v>
+      </c>
+      <c r="N54" s="5" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="55" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A55" t="s">
-        <v>46</v>
+        <v>96</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="C55" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="D55">
-        <f>MONTH(E55&amp;1)</f>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E55" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
       <c r="G55" t="s">
-        <v>111</v>
+        <v>98</v>
       </c>
       <c r="H55" t="s">
-        <v>112</v>
+        <v>255</v>
+      </c>
+      <c r="J55">
+        <v>7</v>
+      </c>
+      <c r="K55" t="s">
+        <v>99</v>
       </c>
       <c r="L55">
-        <v>41.383168015451297</v>
+        <v>38.739795000000001</v>
       </c>
       <c r="M55">
-        <v>-71.709573349086796</v>
+        <v>-83.203586999999999</v>
       </c>
       <c r="N55" s="2" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A56" s="4" t="s">
-        <v>287</v>
+        <v>96</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>288</v>
+        <v>218</v>
       </c>
       <c r="C56" s="4" t="s">
-        <v>291</v>
+        <v>179</v>
       </c>
       <c r="D56">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>30</v>
+        <v>84</v>
       </c>
       <c r="F56">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>289</v>
+        <v>180</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="L56">
-        <v>44.370895386532602</v>
-      </c>
-      <c r="M56">
-        <v>-103.728699130772</v>
-      </c>
-      <c r="N56" s="2" t="s">
-        <v>290</v>
+        <v>181</v>
+      </c>
+      <c r="I56" s="4"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="L56" s="4">
+        <v>41.224018000000001</v>
+      </c>
+      <c r="M56" s="4">
+        <v>-81.510507000000004</v>
+      </c>
+      <c r="N56" s="5" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A57" t="s">
-        <v>19</v>
+      <c r="A57" s="4" t="s">
+        <v>338</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C57" t="s">
-        <v>22</v>
+        <v>339</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>340</v>
       </c>
       <c r="D57">
-        <f>MONTH(E57&amp;1)</f>
-        <v>3</v>
-      </c>
-      <c r="E57" t="s">
-        <v>21</v>
-      </c>
-      <c r="G57" t="s">
-        <v>23</v>
-      </c>
-      <c r="H57" t="s">
-        <v>259</v>
+        <v>11</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F57">
+        <v>1</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>341</v>
+      </c>
+      <c r="H57" s="4" t="s">
+        <v>342</v>
       </c>
       <c r="L57">
-        <v>35.161427052430398</v>
+        <v>35.8014249104668</v>
       </c>
       <c r="M57">
-        <v>-85.368960195175006</v>
-      </c>
-      <c r="N57" s="5" t="s">
-        <v>252</v>
+        <v>-97.461286318959296</v>
+      </c>
+      <c r="N57" s="8" t="s">
+        <v>343</v>
       </c>
     </row>
     <row r="58" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A58" t="s">
-        <v>19</v>
+      <c r="A58" s="4" t="s">
+        <v>338</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C58" t="s">
-        <v>22</v>
+        <v>339</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>344</v>
       </c>
       <c r="D58">
-        <f>MONTH(E58&amp;1)</f>
-        <v>8</v>
-      </c>
-      <c r="E58" t="s">
-        <v>68</v>
-      </c>
-      <c r="G58" t="s">
-        <v>71</v>
-      </c>
-      <c r="H58" t="s">
-        <v>18</v>
-      </c>
-      <c r="J58">
-        <v>6</v>
-      </c>
-      <c r="K58" t="s">
-        <v>72</v>
+        <v>11</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="F58">
+        <v>2</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="H58" s="4" t="s">
+        <v>346</v>
       </c>
       <c r="L58">
-        <v>35.087218</v>
+        <v>34.450079125989902</v>
       </c>
       <c r="M58">
-        <v>-85.111582999999996</v>
+        <v>-97.200097472110798</v>
       </c>
       <c r="N58" s="2" t="s">
-        <v>73</v>
+        <v>347</v>
       </c>
     </row>
     <row r="59" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A59" t="s">
-        <v>19</v>
+      <c r="A59" s="4" t="s">
+        <v>328</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C59" t="s">
-        <v>114</v>
+        <v>329</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>330</v>
       </c>
       <c r="D59">
-        <f>MONTH(E59&amp;1)</f>
-        <v>11</v>
-      </c>
-      <c r="E59" t="s">
-        <v>102</v>
+        <v>4</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="F59">
-        <v>4</v>
-      </c>
-      <c r="G59" t="s">
-        <v>115</v>
-      </c>
-      <c r="H59" t="s">
-        <v>62</v>
-      </c>
-      <c r="J59">
-        <v>6.5</v>
+        <v>2</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="H59" s="4" t="s">
+        <v>332</v>
       </c>
       <c r="L59">
-        <v>35.181998</v>
+        <v>45.669877680785902</v>
       </c>
       <c r="M59">
-        <v>-85.672781000000001</v>
+        <v>-121.893583077792</v>
       </c>
       <c r="N59" s="2" t="s">
-        <v>116</v>
+        <v>333</v>
       </c>
     </row>
     <row r="60" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A60" t="s">
-        <v>19</v>
+      <c r="A60" s="4" t="s">
+        <v>328</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>221</v>
-      </c>
-      <c r="C60" t="s">
-        <v>22</v>
+        <v>329</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>334</v>
       </c>
       <c r="D60">
-        <v>11</v>
-      </c>
-      <c r="E60" t="s">
-        <v>102</v>
+        <v>10</v>
+      </c>
+      <c r="E60" s="4" t="s">
+        <v>84</v>
       </c>
       <c r="F60">
         <v>3</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="H60" t="s">
-        <v>123</v>
-      </c>
-      <c r="J60">
-        <v>5</v>
+        <v>335</v>
+      </c>
+      <c r="H60" s="4" t="s">
+        <v>336</v>
       </c>
       <c r="L60">
-        <v>35.132576999999998</v>
+        <v>42.905827786978001</v>
       </c>
       <c r="M60">
-        <v>-85.419156999999998</v>
+        <v>-122.445547530041</v>
       </c>
       <c r="N60" s="2" t="s">
-        <v>124</v>
+        <v>337</v>
       </c>
     </row>
     <row r="61" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A61" t="s">
-        <v>9</v>
+        <v>66</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C61" t="s">
-        <v>10</v>
+        <v>67</v>
       </c>
       <c r="D61">
         <f>MONTH(E61&amp;1)</f>
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E61" t="s">
-        <v>11</v>
+        <v>68</v>
       </c>
       <c r="G61" t="s">
-        <v>12</v>
+        <v>69</v>
       </c>
       <c r="H61" t="s">
-        <v>13</v>
+        <v>27</v>
+      </c>
+      <c r="J61">
+        <v>9</v>
       </c>
       <c r="L61">
-        <v>29.270030751418901</v>
+        <v>41.345925000000001</v>
       </c>
       <c r="M61">
-        <v>-103.75738789356799</v>
-      </c>
-      <c r="N61" t="s">
-        <v>231</v>
+        <v>-79.218463</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="62" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="C62" t="s">
-        <v>65</v>
+        <v>90</v>
       </c>
       <c r="D62">
         <f>MONTH(E62&amp;1)</f>
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E62" t="s">
-        <v>52</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>232</v>
-      </c>
-      <c r="H62" s="4" t="s">
-        <v>27</v>
+        <v>84</v>
+      </c>
+      <c r="G62" t="s">
+        <v>91</v>
+      </c>
+      <c r="H62" t="s">
+        <v>54</v>
+      </c>
+      <c r="J62">
+        <v>9</v>
       </c>
       <c r="L62">
-        <v>40.651711489342503</v>
+        <v>41.363957999999997</v>
       </c>
       <c r="M62">
-        <v>-111.505570317121</v>
-      </c>
-      <c r="N62" t="s">
-        <v>233</v>
+        <v>-77.356221000000005</v>
+      </c>
+      <c r="N62" s="2" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A63" s="4" t="s">
-        <v>278</v>
+      <c r="A63" t="s">
+        <v>66</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="C63" s="4" t="s">
-        <v>280</v>
+        <v>219</v>
+      </c>
+      <c r="C63" t="s">
+        <v>79</v>
       </c>
       <c r="D63">
-        <v>7</v>
-      </c>
-      <c r="E63" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="F63">
-        <v>2</v>
-      </c>
-      <c r="G63" s="4" t="s">
-        <v>281</v>
-      </c>
-      <c r="H63" s="4" t="s">
-        <v>282</v>
+        <f>MONTH(E63&amp;1)</f>
+        <v>9</v>
+      </c>
+      <c r="E63" t="s">
+        <v>76</v>
+      </c>
+      <c r="G63" t="s">
+        <v>80</v>
+      </c>
+      <c r="H63" t="s">
+        <v>256</v>
+      </c>
+      <c r="J63">
+        <v>9</v>
       </c>
       <c r="L63">
-        <v>47.292665814386503</v>
+        <v>41.134135000000001</v>
       </c>
       <c r="M63">
-        <v>-120.399919279759</v>
+        <v>-77.420109999999994</v>
       </c>
       <c r="N63" s="2" t="s">
-        <v>277</v>
+        <v>81</v>
       </c>
     </row>
     <row r="64" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A64" t="s">
-        <v>35</v>
+      <c r="A64" s="4" t="s">
+        <v>66</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>268</v>
-      </c>
-      <c r="C64" t="s">
-        <v>36</v>
+        <v>219</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>355</v>
       </c>
       <c r="D64">
-        <f>MONTH(E64&amp;1)</f>
+        <v>3</v>
+      </c>
+      <c r="E64" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F64">
         <v>5</v>
       </c>
-      <c r="E64" t="s">
-        <v>30</v>
-      </c>
-      <c r="G64" t="s">
-        <v>37</v>
-      </c>
-      <c r="H64" t="s">
-        <v>38</v>
-      </c>
-      <c r="L64" s="4">
-        <v>42.821545273956801</v>
+      <c r="G64" s="4" t="s">
+        <v>356</v>
+      </c>
+      <c r="H64" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="L64">
+        <v>40.731892037339698</v>
       </c>
       <c r="M64">
-        <v>-88.600563748783202</v>
+        <v>-80.337769738058498</v>
       </c>
       <c r="N64" s="2" t="s">
-        <v>39</v>
+        <v>358</v>
       </c>
     </row>
     <row r="65" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A65" s="4" t="s">
-        <v>324</v>
+        <v>66</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>325</v>
+        <v>219</v>
       </c>
       <c r="C65" s="4" t="s">
-        <v>328</v>
+        <v>375</v>
       </c>
       <c r="D65">
+        <v>4</v>
+      </c>
+      <c r="E65" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="H65" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="L65">
+        <v>40.002812782588997</v>
+      </c>
+      <c r="M65">
+        <v>-77.325546504563803</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A66" t="s">
+        <v>46</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C66" t="s">
+        <v>47</v>
+      </c>
+      <c r="D66">
+        <f>MONTH(E66&amp;1)</f>
         <v>6</v>
       </c>
-      <c r="E65" s="4" t="s">
+      <c r="E66" t="s">
         <v>42</v>
       </c>
-      <c r="F65">
+      <c r="G66" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="H66" t="s">
+        <v>49</v>
+      </c>
+      <c r="L66" s="4">
+        <v>41.441013820781301</v>
+      </c>
+      <c r="M66">
+        <v>-71.463694190880901</v>
+      </c>
+      <c r="N66" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A67" t="s">
+        <v>46</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C67" t="s">
+        <v>110</v>
+      </c>
+      <c r="D67">
+        <f>MONTH(E67&amp;1)</f>
+        <v>11</v>
+      </c>
+      <c r="E67" t="s">
+        <v>102</v>
+      </c>
+      <c r="G67" t="s">
+        <v>111</v>
+      </c>
+      <c r="H67" t="s">
+        <v>112</v>
+      </c>
+      <c r="L67">
+        <v>41.383168015451297</v>
+      </c>
+      <c r="M67">
+        <v>-71.709573349086796</v>
+      </c>
+      <c r="N67" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A68" t="s">
+        <v>46</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="C68" t="s">
+        <v>93</v>
+      </c>
+      <c r="D68">
+        <f>MONTH(E68&amp;1)</f>
+        <v>10</v>
+      </c>
+      <c r="E68" t="s">
+        <v>84</v>
+      </c>
+      <c r="G68" t="s">
+        <v>94</v>
+      </c>
+      <c r="H68" t="s">
+        <v>95</v>
+      </c>
+      <c r="L68">
+        <v>41.361185752662699</v>
+      </c>
+      <c r="M68">
+        <v>-71.4813502625707</v>
+      </c>
+      <c r="N68" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A69" s="4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>286</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="D69">
+        <v>5</v>
+      </c>
+      <c r="E69" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F69">
+        <v>5</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>287</v>
+      </c>
+      <c r="H69" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="L69">
+        <v>44.370895386532602</v>
+      </c>
+      <c r="M69">
+        <v>-103.728699130772</v>
+      </c>
+      <c r="N69" s="2" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A70" t="s">
+        <v>19</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C70" t="s">
+        <v>22</v>
+      </c>
+      <c r="D70">
+        <f>MONTH(E70&amp;1)</f>
+        <v>8</v>
+      </c>
+      <c r="E70" t="s">
+        <v>68</v>
+      </c>
+      <c r="G70" t="s">
+        <v>71</v>
+      </c>
+      <c r="H70" t="s">
+        <v>18</v>
+      </c>
+      <c r="J70">
+        <v>6</v>
+      </c>
+      <c r="K70" t="s">
+        <v>72</v>
+      </c>
+      <c r="L70">
+        <v>35.087218</v>
+      </c>
+      <c r="M70">
+        <v>-85.111582999999996</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A71" t="s">
+        <v>19</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C71" t="s">
+        <v>22</v>
+      </c>
+      <c r="D71">
+        <f>MONTH(E71&amp;1)</f>
+        <v>3</v>
+      </c>
+      <c r="E71" t="s">
+        <v>21</v>
+      </c>
+      <c r="G71" t="s">
+        <v>23</v>
+      </c>
+      <c r="H71" t="s">
+        <v>257</v>
+      </c>
+      <c r="L71">
+        <v>35.161427052430398</v>
+      </c>
+      <c r="M71">
+        <v>-85.368960195175006</v>
+      </c>
+      <c r="N71" s="5" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A72" t="s">
+        <v>19</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s">
+        <v>114</v>
+      </c>
+      <c r="D72">
+        <f>MONTH(E72&amp;1)</f>
+        <v>11</v>
+      </c>
+      <c r="E72" t="s">
+        <v>102</v>
+      </c>
+      <c r="F72">
         <v>4</v>
       </c>
-      <c r="G65" s="4" t="s">
-        <v>327</v>
-      </c>
-      <c r="H65" s="4" t="s">
-        <v>329</v>
-      </c>
-      <c r="L65">
-        <v>46.913974694365898</v>
-      </c>
-      <c r="M65">
-        <v>-103.52377003853699</v>
-      </c>
-      <c r="N65" s="2" t="s">
-        <v>326</v>
+      <c r="G72" t="s">
+        <v>115</v>
+      </c>
+      <c r="H72" t="s">
+        <v>62</v>
+      </c>
+      <c r="J72">
+        <v>6.5</v>
+      </c>
+      <c r="L72">
+        <v>35.181998</v>
+      </c>
+      <c r="M72">
+        <v>-85.672781000000001</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A73" t="s">
+        <v>19</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="C73" t="s">
+        <v>22</v>
+      </c>
+      <c r="D73">
+        <v>11</v>
+      </c>
+      <c r="E73" t="s">
+        <v>102</v>
+      </c>
+      <c r="F73">
+        <v>3</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H73" t="s">
+        <v>123</v>
+      </c>
+      <c r="J73">
+        <v>5</v>
+      </c>
+      <c r="L73">
+        <v>35.132576999999998</v>
+      </c>
+      <c r="M73">
+        <v>-85.419156999999998</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A74" t="s">
+        <v>9</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C74" t="s">
+        <v>10</v>
+      </c>
+      <c r="D74">
+        <f>MONTH(E74&amp;1)</f>
+        <v>1</v>
+      </c>
+      <c r="E74" t="s">
+        <v>11</v>
+      </c>
+      <c r="G74" t="s">
+        <v>12</v>
+      </c>
+      <c r="H74" t="s">
+        <v>13</v>
+      </c>
+      <c r="L74">
+        <v>29.270030751418901</v>
+      </c>
+      <c r="M74">
+        <v>-103.75738789356799</v>
+      </c>
+      <c r="N74" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A75" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="D75">
+        <v>3</v>
+      </c>
+      <c r="E75" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F75">
+        <v>3</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="H75" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="L75">
+        <v>34.297705212943399</v>
+      </c>
+      <c r="M75">
+        <v>-99.739548228350998</v>
+      </c>
+      <c r="N75" s="5" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A76" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>382</v>
+      </c>
+      <c r="D76">
+        <v>3</v>
+      </c>
+      <c r="E76" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F76">
+        <v>4</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>383</v>
+      </c>
+      <c r="H76" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="L76">
+        <v>30.5080101049764</v>
+      </c>
+      <c r="M76">
+        <v>-98.1048887125487</v>
+      </c>
+      <c r="N76" s="5" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A77" t="s">
+        <v>64</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="C77" t="s">
+        <v>65</v>
+      </c>
+      <c r="D77">
+        <f>MONTH(E77&amp;1)</f>
+        <v>7</v>
+      </c>
+      <c r="E77" t="s">
+        <v>52</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="H77" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="L77">
+        <v>40.651711489342503</v>
+      </c>
+      <c r="M77">
+        <v>-111.505570317121</v>
+      </c>
+      <c r="N77" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A78" s="4" t="s">
+        <v>276</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>277</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>278</v>
+      </c>
+      <c r="D78">
+        <v>7</v>
+      </c>
+      <c r="E78" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="F78">
+        <v>2</v>
+      </c>
+      <c r="G78" s="4" t="s">
+        <v>279</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>280</v>
+      </c>
+      <c r="L78">
+        <v>47.292665814386503</v>
+      </c>
+      <c r="M78">
+        <v>-120.399919279759</v>
+      </c>
+      <c r="N78" s="2" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A79" t="s">
+        <v>35</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>266</v>
+      </c>
+      <c r="C79" t="s">
+        <v>36</v>
+      </c>
+      <c r="D79">
+        <f>MONTH(E79&amp;1)</f>
+        <v>5</v>
+      </c>
+      <c r="E79" t="s">
+        <v>30</v>
+      </c>
+      <c r="G79" t="s">
+        <v>37</v>
+      </c>
+      <c r="H79" t="s">
+        <v>38</v>
+      </c>
+      <c r="L79" s="4">
+        <v>42.821545273956801</v>
+      </c>
+      <c r="M79">
+        <v>-88.600563748783202</v>
+      </c>
+      <c r="N79" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A80" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>385</v>
+      </c>
+      <c r="D80">
+        <v>9</v>
+      </c>
+      <c r="E80" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F80">
+        <v>2</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>386</v>
+      </c>
+      <c r="L80">
+        <v>38.963440766596698</v>
+      </c>
+      <c r="M80">
+        <v>-84.081651159329098</v>
+      </c>
+      <c r="N80" s="2" t="s">
+        <v>387</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="N31" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="N64" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="N9" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="N35" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="N43" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="N50" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="N58" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="N51" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="N52" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="N47" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="N4" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="N36" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N79" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N10" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N37" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N50" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N61" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="N70" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="N63" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="N62" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="N55" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="N3" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
     <hyperlink ref="N34" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="N55" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="N59" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="N26" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="N60" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="N3" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="N12" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="N13" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="N14" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="N67" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="N72" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="N30" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="N73" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="N4" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="N13" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="N14" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="N15" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
     <hyperlink ref="N24" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="N22" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="N23" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="N44" r:id="rId24" xr:uid="{B1E10B24-F054-E547-BD3C-660C0672113E}"/>
-    <hyperlink ref="N6" r:id="rId25" xr:uid="{894ECB44-0541-8248-BBC2-F2EB43D34ADF}"/>
-    <hyperlink ref="N39" r:id="rId26" xr:uid="{2AA9988F-6D01-144B-81DA-87954893D26D}"/>
+    <hyperlink ref="N23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="N25" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="N52" r:id="rId24" xr:uid="{B1E10B24-F054-E547-BD3C-660C0672113E}"/>
+    <hyperlink ref="N8" r:id="rId25" xr:uid="{894ECB44-0541-8248-BBC2-F2EB43D34ADF}"/>
+    <hyperlink ref="N44" r:id="rId26" xr:uid="{2AA9988F-6D01-144B-81DA-87954893D26D}"/>
     <hyperlink ref="N2" r:id="rId27" xr:uid="{C929B912-E898-FB4A-A56C-63AD48FB3C12}"/>
-    <hyperlink ref="N5" r:id="rId28" xr:uid="{E2B0F023-1474-6446-98F1-3AB4FF697C20}"/>
-    <hyperlink ref="N21" r:id="rId29" xr:uid="{D4186AD3-3DB1-1748-BE0E-5237851CE632}"/>
-    <hyperlink ref="N32" r:id="rId30" display="https://ultrasignup.com/register.aspx?did=121875" xr:uid="{D8FE7B00-306C-E843-BBB5-677644870ACC}"/>
-    <hyperlink ref="N33" r:id="rId31" xr:uid="{AE57CCA9-648D-F54A-A2BF-9CDA9126A94E}"/>
-    <hyperlink ref="N48" r:id="rId32" xr:uid="{D7230747-A69F-AA4A-96F8-7DE9C9C4A60B}"/>
-    <hyperlink ref="N49" r:id="rId33" xr:uid="{7F4BFEFD-5AD7-8C40-8BDC-4D42308FFEB7}"/>
-    <hyperlink ref="N57" r:id="rId34" display="https://www.badbeardevents.com/featured-races/stump-jump-50k-and-10-miler" xr:uid="{B6E400ED-9EF0-FC43-921D-CEBB3BD2D97E}"/>
-    <hyperlink ref="M27" r:id="rId35" display="https://www.google.com/maps/place/38%C2%B011'28.8%22N+83%C2%B025'53.1%22W/@38.1913353,-83.4325027,427m/data=!3m2!1e3!4b1!4m4!3m3!8m2!3d38.1913335!4d-83.4314201!5m1!1e1?entry=ttu&amp;g_ep=EgoyMDI1MDQxNi4xIKXMDSoASAFQAw%3D%3D" xr:uid="{075506EC-582D-5C4E-A0FF-0E65726F3261}"/>
-    <hyperlink ref="L27" r:id="rId36" display="https://www.google.com/maps/place/38%C2%B011'28.8%22N+83%C2%B025'53.1%22W/@38.1913353,-83.4325027,427m/data=!3m2!1e3!4b1!4m4!3m3!8m2!3d38.1913335!4d-83.4314201!5m1!1e1?entry=ttu&amp;g_ep=EgoyMDI1MDQxNi4xIKXMDSoASAFQAw%3D%3D" xr:uid="{47D09849-195F-B74C-84AE-230308A58C81}"/>
+    <hyperlink ref="N9" r:id="rId28" xr:uid="{E2B0F023-1474-6446-98F1-3AB4FF697C20}"/>
+    <hyperlink ref="N26" r:id="rId29" xr:uid="{D4186AD3-3DB1-1748-BE0E-5237851CE632}"/>
+    <hyperlink ref="N33" r:id="rId30" xr:uid="{AE57CCA9-648D-F54A-A2BF-9CDA9126A94E}"/>
+    <hyperlink ref="N56" r:id="rId31" xr:uid="{D7230747-A69F-AA4A-96F8-7DE9C9C4A60B}"/>
+    <hyperlink ref="N54" r:id="rId32" xr:uid="{7F4BFEFD-5AD7-8C40-8BDC-4D42308FFEB7}"/>
+    <hyperlink ref="M28" r:id="rId33" display="https://www.google.com/maps/place/38%C2%B011'28.8%22N+83%C2%B025'53.1%22W/@38.1913353,-83.4325027,427m/data=!3m2!1e3!4b1!4m4!3m3!8m2!3d38.1913335!4d-83.4314201!5m1!1e1?entry=ttu&amp;g_ep=EgoyMDI1MDQxNi4xIKXMDSoASAFQAw%3D%3D" xr:uid="{075506EC-582D-5C4E-A0FF-0E65726F3261}"/>
+    <hyperlink ref="L28" r:id="rId34" display="https://www.google.com/maps/place/38%C2%B011'28.8%22N+83%C2%B025'53.1%22W/@38.1913353,-83.4325027,427m/data=!3m2!1e3!4b1!4m4!3m3!8m2!3d38.1913335!4d-83.4314201!5m1!1e1?entry=ttu&amp;g_ep=EgoyMDI1MDQxNi4xIKXMDSoASAFQAw%3D%3D" xr:uid="{47D09849-195F-B74C-84AE-230308A58C81}"/>
+    <hyperlink ref="N18" r:id="rId35" xr:uid="{149B1691-ADF9-1E4C-AF69-D26286ADA2A0}"/>
+    <hyperlink ref="N75" r:id="rId36" xr:uid="{0EDD11A3-E6C2-8648-984B-32C0F1E3C2F4}"/>
+    <hyperlink ref="N76" r:id="rId37" xr:uid="{35B31226-CE4C-1D4F-99CA-BEF8E7C708D8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
-    <tablePart r:id="rId37"/>
+    <tablePart r:id="rId38"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>